<commit_message>
Regenerate October against the merged export: 335 flights, 10 Oct filled
Top-level FR data.zip deduplicated to 1,083 unique tracks
(sha256 a60990fd...); October month zip rebuilt to 335 UR tracks
(a6add0e2...); September zip untouched. Pipeline rerun
(rebuild_month -> build_october_fta -> rebuild_month ->
build_conditions -> build_od_matrix_october): 335 flights, 330 with
tails, 113 triangle sectors. FTA cross-check improves to 324/354 legs
matched (was 306) and 30 without a track (was 48) - the 18 new tracks
cover 10 Oct, which is no longer a blackout; data_gaps.md,
schedule_delays.md, punctuality.md scoreboard (117 early / 104 on
time / 85 delayed / 18 heavily delayed of 324), runway/weather/
triangle write-ups and the OD matrices (Oct 10 now 17 sectors)
updated to match. Stale '10 Oct empty/blackout' text removed from
work/build_october_fta.py and work/build_od_matrix_october.py.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UR OCTOBER 2026/od_matrix_october2026.xlsx
+++ b/UR OCTOBER 2026/od_matrix_october2026.xlsx
@@ -483,7 +483,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Coverage 1-16 Oct 2026 (track export window). 10 Oct: no recorded departures — see PDF.</t>
+          <t>Coverage 1-16 Oct 2026 (track export window).</t>
         </is>
       </c>
     </row>
@@ -1301,7 +1301,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>2026-10-09 — 25 sectors</t>
+          <t>2026-10-09 — 26 sectors</t>
         </is>
       </c>
     </row>
@@ -1526,8 +1526,11 @@
           <t>LGW</t>
         </is>
       </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -1609,7 +1612,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>1</v>
@@ -1654,7 +1657,7 @@
         <v>1</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -1693,7 +1696,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>2026-10-10 — 0 sectors (no recorded departures)</t>
+          <t>2026-10-10 — 17 sectors</t>
         </is>
       </c>
     </row>
@@ -1790,8 +1793,32 @@
           <t>EBB</t>
         </is>
       </c>
+      <c r="D4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>2</v>
+      </c>
       <c r="Q4" s="5" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
     </row>
     <row r="5">
@@ -1820,8 +1847,11 @@
           <t>DAR</t>
         </is>
       </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q7" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -1830,8 +1860,11 @@
           <t>HRE</t>
         </is>
       </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q8" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -1840,8 +1873,11 @@
           <t>JNB</t>
         </is>
       </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q9" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10">
@@ -1860,8 +1896,11 @@
           <t>JUB</t>
         </is>
       </c>
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q11" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -1880,8 +1919,11 @@
           <t>LOS</t>
         </is>
       </c>
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q13" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -1890,8 +1932,11 @@
           <t>LUN</t>
         </is>
       </c>
+      <c r="B14" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q14" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -1910,8 +1955,11 @@
           <t>MGQ</t>
         </is>
       </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q16" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -1920,8 +1968,11 @@
           <t>NBO</t>
         </is>
       </c>
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q17" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -1941,28 +1992,28 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J19" s="5" t="n">
         <v>0</v>
@@ -1971,22 +2022,22 @@
         <v>0</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="P19" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
@@ -4310,7 +4361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D266"/>
+  <dimension ref="A1:D283"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7443,7 +7494,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
@@ -7463,7 +7514,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -7483,7 +7534,7 @@
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
@@ -7503,7 +7554,7 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
@@ -7512,18 +7563,18 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-09</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -7532,18 +7583,18 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -7558,17 +7609,17 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="D163" t="n">
@@ -7578,17 +7629,17 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
           <t>DAR</t>
-        </is>
-      </c>
-      <c r="C164" t="inlineStr">
-        <is>
-          <t>NBO</t>
         </is>
       </c>
       <c r="D164" t="n">
@@ -7598,7 +7649,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -7608,7 +7659,7 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="D165" t="n">
@@ -7618,7 +7669,7 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -7628,7 +7679,7 @@
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D166" t="n">
@@ -7638,7 +7689,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -7648,7 +7699,7 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D167" t="n">
@@ -7658,7 +7709,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -7668,7 +7719,7 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="D168" t="n">
@@ -7678,7 +7729,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -7688,7 +7739,7 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>LGW</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="D169" t="n">
@@ -7698,7 +7749,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -7708,27 +7759,27 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -7738,17 +7789,17 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D172" t="n">
@@ -7758,17 +7809,17 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D173" t="n">
@@ -7778,37 +7829,37 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>ZNZ</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D175" t="n">
@@ -7818,12 +7869,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -7838,12 +7889,12 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-10-11</t>
+          <t>2026-10-10</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>JRO</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
@@ -7863,7 +7914,7 @@
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -7883,7 +7934,7 @@
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -7903,7 +7954,7 @@
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
@@ -7923,32 +7974,32 @@
       </c>
       <c r="B181" t="inlineStr">
         <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
           <t>NBO</t>
         </is>
       </c>
-      <c r="C181" t="inlineStr">
-        <is>
-          <t>EBB</t>
-        </is>
-      </c>
       <c r="D181" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
           <t>BJM</t>
-        </is>
-      </c>
-      <c r="C182" t="inlineStr">
-        <is>
-          <t>EBB</t>
         </is>
       </c>
       <c r="D182" t="n">
@@ -7958,27 +8009,27 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
           <t>DAR</t>
         </is>
       </c>
-      <c r="C183" t="inlineStr">
-        <is>
-          <t>EBB</t>
-        </is>
-      </c>
       <c r="D183" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -7988,7 +8039,7 @@
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D184" t="n">
@@ -7998,7 +8049,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -8008,17 +8059,17 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -8028,17 +8079,17 @@
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="D186" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -8048,7 +8099,7 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="D187" t="n">
@@ -8058,7 +8109,7 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -8068,7 +8119,7 @@
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="D188" t="n">
@@ -8078,7 +8129,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -8088,7 +8139,7 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="D189" t="n">
@@ -8098,7 +8149,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -8108,62 +8159,62 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>ZNZ</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
@@ -8178,12 +8229,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>JRO</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -8198,17 +8249,17 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D195" t="n">
@@ -8218,12 +8269,12 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-10-12</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
@@ -8232,18 +8283,18 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -8258,12 +8309,12 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-11</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C198" t="inlineStr">
@@ -8272,23 +8323,23 @@
         </is>
       </c>
       <c r="D198" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D199" t="n">
@@ -8298,27 +8349,27 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C200" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D200" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -8328,7 +8379,7 @@
       </c>
       <c r="C201" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="D201" t="n">
@@ -8338,7 +8389,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -8348,17 +8399,17 @@
       </c>
       <c r="C202" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="D202" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -8368,17 +8419,17 @@
       </c>
       <c r="C203" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D203" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -8388,7 +8439,7 @@
       </c>
       <c r="C204" t="inlineStr">
         <is>
-          <t>LGW</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D204" t="n">
@@ -8398,7 +8449,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -8408,7 +8459,7 @@
       </c>
       <c r="C205" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="D205" t="n">
@@ -8418,7 +8469,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -8428,37 +8479,37 @@
       </c>
       <c r="C206" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="D206" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D207" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -8468,7 +8519,7 @@
       </c>
       <c r="C208" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D208" t="n">
@@ -8478,7 +8529,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -8492,13 +8543,13 @@
         </is>
       </c>
       <c r="D209" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -8508,7 +8559,7 @@
       </c>
       <c r="C210" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D210" t="n">
@@ -8518,12 +8569,12 @@
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B211" t="inlineStr">
         <is>
-          <t>LGW</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="C211" t="inlineStr">
@@ -8538,7 +8589,7 @@
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B212" t="inlineStr">
@@ -8548,7 +8599,7 @@
       </c>
       <c r="C212" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="D212" t="n">
@@ -8558,12 +8609,12 @@
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>2026-10-13</t>
+          <t>2026-10-12</t>
         </is>
       </c>
       <c r="B213" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C213" t="inlineStr">
@@ -8572,7 +8623,7 @@
         </is>
       </c>
       <c r="D213" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="214">
@@ -8583,7 +8634,7 @@
       </c>
       <c r="B214" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C214" t="inlineStr">
@@ -8592,18 +8643,18 @@
         </is>
       </c>
       <c r="D214" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B215" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C215" t="inlineStr">
@@ -8618,7 +8669,7 @@
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B216" t="inlineStr">
@@ -8638,7 +8689,7 @@
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B217" t="inlineStr">
@@ -8648,7 +8699,7 @@
       </c>
       <c r="C217" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="D217" t="n">
@@ -8658,7 +8709,7 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B218" t="inlineStr">
@@ -8668,7 +8719,7 @@
       </c>
       <c r="C218" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="D218" t="n">
@@ -8678,7 +8729,7 @@
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B219" t="inlineStr">
@@ -8688,7 +8739,7 @@
       </c>
       <c r="C219" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D219" t="n">
@@ -8698,7 +8749,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B220" t="inlineStr">
@@ -8708,7 +8759,7 @@
       </c>
       <c r="C220" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D220" t="n">
@@ -8718,7 +8769,7 @@
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B221" t="inlineStr">
@@ -8728,7 +8779,7 @@
       </c>
       <c r="C221" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="D221" t="n">
@@ -8738,7 +8789,7 @@
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B222" t="inlineStr">
@@ -8748,7 +8799,7 @@
       </c>
       <c r="C222" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="D222" t="n">
@@ -8758,7 +8809,7 @@
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B223" t="inlineStr">
@@ -8778,17 +8829,17 @@
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B224" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="C224" t="inlineStr">
         <is>
-          <t>ZNZ</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D224" t="n">
@@ -8798,7 +8849,7 @@
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B225" t="inlineStr">
@@ -8818,7 +8869,7 @@
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B226" t="inlineStr">
@@ -8832,23 +8883,23 @@
         </is>
       </c>
       <c r="D226" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B227" t="inlineStr">
         <is>
-          <t>JRO</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="C227" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D227" t="n">
@@ -8858,12 +8909,12 @@
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B228" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="C228" t="inlineStr">
@@ -8878,7 +8929,7 @@
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B229" t="inlineStr">
@@ -8898,12 +8949,12 @@
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B230" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="C230" t="inlineStr">
@@ -8918,7 +8969,7 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>2026-10-14</t>
+          <t>2026-10-13</t>
         </is>
       </c>
       <c r="B231" t="inlineStr">
@@ -8932,7 +8983,7 @@
         </is>
       </c>
       <c r="D231" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="232">
@@ -8943,12 +8994,12 @@
       </c>
       <c r="B232" t="inlineStr">
         <is>
-          <t>ZNZ</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C232" t="inlineStr">
         <is>
-          <t>JRO</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D232" t="n">
@@ -8958,17 +9009,17 @@
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B233" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
           <t>BJM</t>
-        </is>
-      </c>
-      <c r="C233" t="inlineStr">
-        <is>
-          <t>EBB</t>
         </is>
       </c>
       <c r="D233" t="n">
@@ -8978,17 +9029,17 @@
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B234" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
           <t>BOM</t>
-        </is>
-      </c>
-      <c r="C234" t="inlineStr">
-        <is>
-          <t>EBB</t>
         </is>
       </c>
       <c r="D234" t="n">
@@ -8998,17 +9049,17 @@
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B235" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
           <t>DAR</t>
-        </is>
-      </c>
-      <c r="C235" t="inlineStr">
-        <is>
-          <t>EBB</t>
         </is>
       </c>
       <c r="D235" t="n">
@@ -9018,7 +9069,7 @@
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B236" t="inlineStr">
@@ -9028,7 +9079,7 @@
       </c>
       <c r="C236" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="D236" t="n">
@@ -9038,7 +9089,7 @@
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B237" t="inlineStr">
@@ -9048,7 +9099,7 @@
       </c>
       <c r="C237" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D237" t="n">
@@ -9058,7 +9109,7 @@
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B238" t="inlineStr">
@@ -9068,7 +9119,7 @@
       </c>
       <c r="C238" t="inlineStr">
         <is>
-          <t>HRE</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D238" t="n">
@@ -9078,7 +9129,7 @@
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B239" t="inlineStr">
@@ -9088,7 +9139,7 @@
       </c>
       <c r="C239" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="D239" t="n">
@@ -9098,7 +9149,7 @@
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B240" t="inlineStr">
@@ -9108,17 +9159,17 @@
       </c>
       <c r="C240" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D240" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -9128,7 +9179,7 @@
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>ZNZ</t>
         </is>
       </c>
       <c r="D241" t="n">
@@ -9138,32 +9189,32 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="D242" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="C243" t="inlineStr">
@@ -9172,18 +9223,18 @@
         </is>
       </c>
       <c r="D243" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>JRO</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
@@ -9198,12 +9249,12 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
@@ -9212,18 +9263,18 @@
         </is>
       </c>
       <c r="D245" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
@@ -9238,12 +9289,12 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
@@ -9258,17 +9309,17 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>BJM</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D248" t="n">
@@ -9278,17 +9329,17 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-14</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>ZNZ</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>JRO</t>
         </is>
       </c>
       <c r="D249" t="n">
@@ -9298,17 +9349,17 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D250" t="n">
@@ -9318,17 +9369,17 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D251" t="n">
@@ -9338,17 +9389,17 @@
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>LGW</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D252" t="n">
@@ -9358,7 +9409,7 @@
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B253" t="inlineStr">
@@ -9368,7 +9419,7 @@
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="D253" t="n">
@@ -9378,7 +9429,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B254" t="inlineStr">
@@ -9388,7 +9439,7 @@
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>LUN</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="D254" t="n">
@@ -9398,7 +9449,7 @@
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B255" t="inlineStr">
@@ -9408,7 +9459,7 @@
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>HRE</t>
         </is>
       </c>
       <c r="D255" t="n">
@@ -9418,7 +9469,7 @@
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B256" t="inlineStr">
@@ -9428,7 +9479,7 @@
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D256" t="n">
@@ -9438,7 +9489,7 @@
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B257" t="inlineStr">
@@ -9448,17 +9499,17 @@
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D257" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B258" t="inlineStr">
@@ -9468,7 +9519,7 @@
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>ZNZ</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="D258" t="n">
@@ -9478,17 +9529,17 @@
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>JNB</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="D259" t="n">
@@ -9498,12 +9549,12 @@
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>JRO</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
@@ -9518,12 +9569,12 @@
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>JUB</t>
+          <t>LUN</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
@@ -9538,12 +9589,12 @@
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>2026-10-16</t>
+          <t>2026-10-15</t>
         </is>
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>NBO</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
@@ -9552,7 +9603,7 @@
         </is>
       </c>
       <c r="D262" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="263">
@@ -9563,7 +9614,7 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
@@ -9583,7 +9634,7 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
@@ -9603,16 +9654,16 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="D265" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="266">
@@ -9623,15 +9674,355 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="D266" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="D267" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="D268" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="D269" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="D270" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="D271" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="D272" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="D273" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="D274" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
           <t>ZNZ</t>
         </is>
       </c>
-      <c r="C266" t="inlineStr">
+      <c r="D275" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D276" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
         <is>
           <t>JRO</t>
         </is>
       </c>
-      <c r="D266" t="n">
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D277" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D278" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D279" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D280" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D281" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D282" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10038,19 +10429,19 @@
         <v>14</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>16</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>15</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>7</v>
@@ -10059,22 +10450,22 @@
         <v>10</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>152</v>
+        <v>161</v>
       </c>
     </row>
     <row r="5">
@@ -10110,13 +10501,13 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="8">
@@ -10126,13 +10517,13 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="9">
@@ -10142,10 +10533,10 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10">
@@ -10168,13 +10559,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="O11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="12">
@@ -10184,10 +10575,10 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13">
@@ -10197,10 +10588,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14">
@@ -10210,13 +10601,13 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="15">
@@ -10239,10 +10630,10 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="17">
@@ -10252,10 +10643,10 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="18">
@@ -10278,28 +10669,28 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>14</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J19" s="5" t="n">
         <v>7</v>
@@ -10308,22 +10699,22 @@
         <v>10</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>7</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="P19" s="5" t="n">
         <v>7</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>317</v>
+        <v>335</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cascade 2026-10-20 export: dedupe 1,143 -> 1,108 tracks, extend October to 18th
Top-level FR data.zip deduped by content (35 duplicates removed,
sha256 ebdff074...); all 1,083 previous tracks retained, 25 new UR
tracks (1 on 16 Oct - the missing UR111 return; 16 on 17 Oct, 8 on 18 Oct).
October month zip rebuilt to 360 UR tracks (151,068 fixes, sha256
01781f80...).

FTA plans for 17-18 Oct transcribed (work/fta_oct2026.csv, 402 operating
legs); October pipeline rerun (360 flights, 356 tailed, 120 triangle
sectors, 351 FTA-matched, 40 no-track legs + 11 at/after export end).
HUEN METAR extended to 19 Oct (metar/HUEN_202610_part3.csv); conditions
rebuilt (360 rows, 343 with an EBB-end report). Daily OD matrices
regenerated for 1-18 Oct (306 tidy rows, EBB 175 out / 169 in).
Two CANCELLED Mogadishu legs (17 Oct) are no longer counted as gaps.
Docs updated throughout.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UR OCTOBER 2026/od_matrix_october2026.xlsx
+++ b/UR OCTOBER 2026/od_matrix_october2026.xlsx
@@ -26,7 +26,9 @@
     <sheet name="2026-10-14" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-10-15" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="2026-10-16" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet name="DIVERSION_CHECK" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-10-17" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="2026-10-18" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="DIVERSION_CHECK" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -483,7 +485,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Coverage 1-16 Oct 2026 (track export window).</t>
+          <t>Coverage 1-18 Oct 2026 (track export window).</t>
         </is>
       </c>
     </row>
@@ -3991,7 +3993,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>2026-10-16 — 25 sectors</t>
+          <t>2026-10-16 — 26 sectors</t>
         </is>
       </c>
     </row>
@@ -4216,8 +4218,11 @@
           <t>LGW</t>
         </is>
       </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -4302,7 +4307,7 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>1</v>
@@ -4347,7 +4352,7 @@
         <v>1</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -4361,7 +4366,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D283"/>
+  <dimension ref="A1:D307"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9934,7 +9939,7 @@
       </c>
       <c r="B279" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="C279" t="inlineStr">
@@ -9954,7 +9959,7 @@
       </c>
       <c r="B280" t="inlineStr">
         <is>
-          <t>MBA</t>
+          <t>LOS</t>
         </is>
       </c>
       <c r="C280" t="inlineStr">
@@ -9974,7 +9979,7 @@
       </c>
       <c r="B281" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>MBA</t>
         </is>
       </c>
       <c r="C281" t="inlineStr">
@@ -9994,7 +9999,7 @@
       </c>
       <c r="B282" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>MGQ</t>
         </is>
       </c>
       <c r="C282" t="inlineStr">
@@ -10003,7 +10008,7 @@
         </is>
       </c>
       <c r="D282" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="283">
@@ -10014,15 +10019,495 @@
       </c>
       <c r="B283" t="inlineStr">
         <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D283" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>2026-10-16</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
           <t>ZNZ</t>
         </is>
       </c>
-      <c r="C283" t="inlineStr">
+      <c r="C284" t="inlineStr">
         <is>
           <t>JRO</t>
         </is>
       </c>
-      <c r="D283" t="n">
+      <c r="D284" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D285" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="D286" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="D287" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="D288" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="D289" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="D290" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="D291" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="D292" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D293" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D294" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D295" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D296" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D297" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>2026-10-17</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D298" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D299" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D300" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="D301" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="D302" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="D303" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="D304" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="D305" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="D306" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
         <v>1</v>
       </c>
     </row>
@@ -10032,6 +10517,739 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-17 — 15 sectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>from \ to</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL IN</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>7</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>15</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-18 — 9 sectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>from \ to</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL IN</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>3</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>9</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10328,7 +11546,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>October 2026 (1-16 Oct) — all sectors</t>
+          <t>October 2026 (1-18 Oct) — all sectors</t>
         </is>
       </c>
     </row>
@@ -10429,43 +11647,43 @@
         <v>14</v>
       </c>
       <c r="D4" s="4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>17</v>
       </c>
-      <c r="F4" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>18</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>16</v>
-      </c>
       <c r="J4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>10</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>9</v>
       </c>
       <c r="M4" s="4" t="n">
         <v>7</v>
       </c>
       <c r="N4" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>34</v>
+        <v>37</v>
       </c>
       <c r="P4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="5">
@@ -10488,10 +11706,10 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q6" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="7">
@@ -10501,13 +11719,13 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
@@ -10517,13 +11735,13 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -10533,10 +11751,10 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
@@ -10559,13 +11777,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="O11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="12">
@@ -10575,10 +11793,10 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -10588,10 +11806,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="14">
@@ -10601,13 +11819,13 @@
         </is>
       </c>
       <c r="B14" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>3</v>
       </c>
       <c r="Q14" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -10643,10 +11861,10 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>37</v>
+        <v>39</v>
       </c>
     </row>
     <row r="18">
@@ -10669,52 +11887,52 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>158</v>
+        <v>169</v>
       </c>
       <c r="C19" s="5" t="n">
         <v>14</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I19" s="5" t="n">
+        <v>17</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>8</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>11</v>
+      </c>
+      <c r="L19" s="5" t="n">
         <v>16</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="L19" s="5" t="n">
-        <v>15</v>
       </c>
       <c r="M19" s="5" t="n">
         <v>7</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="P19" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>335</v>
+        <v>360</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Cascade main's new export (work/FR data.zip @fece7ad): October to 19th
New export on main is a strict superset of the branch archive:
1,133 unique tracks (+25, none lost) - 17 tracks filling the
18 Oct afternoon/evening and 8 on the 19 Oct morning. Top-level
FR data.zip replaced deduped (sha256 9590df76...), October month
zip rebuilt to 385 UR tracks (161,295 fixes, sha256 35457367...).

FTA plan for 19 Oct transcribed (AMENDED plan, 20 legs): 422 legs
total, 377 matched, 35 without a track, 10 unverifiable at the new
export end (last fix 19 Oct 12:02Z). Full October cascade rerun
(385 flights, 381 tailed, 129 triangle sectors, conditions, 19
daily OD matrices / 325 tidy rows) and October docs refreshed.
Website data.json regenerated: 1,007 flights, header now 1 Sep -
19 Oct 2026.

Co-authored-by: arena-agent <297053741+arena-agent@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/UR OCTOBER 2026/od_matrix_october2026.xlsx
+++ b/UR OCTOBER 2026/od_matrix_october2026.xlsx
@@ -28,7 +28,8 @@
     <sheet name="2026-10-16" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="2026-10-17" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="2026-10-18" sheetId="21" state="visible" r:id="rId21"/>
-    <sheet name="DIVERSION_CHECK" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="2026-10-19" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet name="DIVERSION_CHECK" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -485,7 +486,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Coverage 1-18 Oct 2026 (track export window).</t>
+          <t>Coverage 1-19 Oct 2026 (track export window).</t>
         </is>
       </c>
     </row>
@@ -4366,7 +4367,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D307"/>
+  <dimension ref="A1:D326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10339,7 +10340,7 @@
       </c>
       <c r="B299" t="inlineStr">
         <is>
-          <t>BOM</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="C299" t="inlineStr">
@@ -10359,7 +10360,7 @@
       </c>
       <c r="B300" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>BOM</t>
         </is>
       </c>
       <c r="C300" t="inlineStr">
@@ -10379,16 +10380,16 @@
       </c>
       <c r="B301" t="inlineStr">
         <is>
-          <t>EBB</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="C301" t="inlineStr">
         <is>
-          <t>DAR</t>
+          <t>EBB</t>
         </is>
       </c>
       <c r="D301" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="302">
@@ -10404,7 +10405,7 @@
       </c>
       <c r="C302" t="inlineStr">
         <is>
-          <t>LGW</t>
+          <t>BJM</t>
         </is>
       </c>
       <c r="D302" t="n">
@@ -10424,7 +10425,7 @@
       </c>
       <c r="C303" t="inlineStr">
         <is>
-          <t>LOS</t>
+          <t>DAR</t>
         </is>
       </c>
       <c r="D303" t="n">
@@ -10444,7 +10445,7 @@
       </c>
       <c r="C304" t="inlineStr">
         <is>
-          <t>MGQ</t>
+          <t>JNB</t>
         </is>
       </c>
       <c r="D304" t="n">
@@ -10464,7 +10465,7 @@
       </c>
       <c r="C305" t="inlineStr">
         <is>
-          <t>NBO</t>
+          <t>JUB</t>
         </is>
       </c>
       <c r="D305" t="n">
@@ -10484,7 +10485,7 @@
       </c>
       <c r="C306" t="inlineStr">
         <is>
-          <t>ZNZ</t>
+          <t>LGW</t>
         </is>
       </c>
       <c r="D306" t="n">
@@ -10499,16 +10500,396 @@
       </c>
       <c r="B307" t="inlineStr">
         <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="D307" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="D308" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="D309" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="D310" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
           <t>NBO</t>
         </is>
       </c>
-      <c r="C307" t="inlineStr">
-        <is>
-          <t>EBB</t>
-        </is>
-      </c>
-      <c r="D307" t="n">
-        <v>1</v>
+      <c r="D311" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="D312" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D313" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D314" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D315" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D316" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D317" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D318" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D319" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="D320" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="D321" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="D322" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="D323" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D324" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D325" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="D326" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>
@@ -10921,7 +11302,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>2026-10-18 — 9 sectors</t>
+          <t>2026-10-18 — 26 sectors</t>
         </is>
       </c>
     </row>
@@ -11018,26 +11399,41 @@
           <t>EBB</t>
         </is>
       </c>
+      <c r="C4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="E4" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="J4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="K4" s="4" t="n">
         <v>1</v>
       </c>
+      <c r="L4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="N4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
@@ -11046,8 +11442,11 @@
           <t>BJM</t>
         </is>
       </c>
+      <c r="B5" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q5" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -11070,10 +11469,10 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8">
@@ -11102,8 +11501,11 @@
           <t>JRO</t>
         </is>
       </c>
+      <c r="B10" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q10" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -11112,8 +11514,11 @@
           <t>JUB</t>
         </is>
       </c>
+      <c r="B11" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q11" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="12">
@@ -11122,8 +11527,11 @@
           <t>LGW</t>
         </is>
       </c>
+      <c r="B12" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q12" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="13">
@@ -11132,8 +11540,11 @@
           <t>LOS</t>
         </is>
       </c>
+      <c r="B13" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q13" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14">
@@ -11152,8 +11563,11 @@
           <t>MBA</t>
         </is>
       </c>
+      <c r="B15" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q15" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="16">
@@ -11162,8 +11576,11 @@
           <t>MGQ</t>
         </is>
       </c>
+      <c r="B16" s="4" t="n">
+        <v>1</v>
+      </c>
       <c r="Q16" s="5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17">
@@ -11173,10 +11590,10 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="18">
@@ -11196,52 +11613,52 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
+        <v>13</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="O19" s="5" t="n">
         <v>3</v>
       </c>
-      <c r="C19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="5" t="n">
-        <v>1</v>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>1</v>
-      </c>
       <c r="P19" s="5" t="n">
         <v>1</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>9</v>
+        <v>26</v>
       </c>
     </row>
   </sheetData>
@@ -11250,6 +11667,359 @@
 </file>
 
 <file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:Q19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="11" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="6" customWidth="1" min="7" max="7"/>
+    <col width="6" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="6" customWidth="1" min="11" max="11"/>
+    <col width="6" customWidth="1" min="12" max="12"/>
+    <col width="6" customWidth="1" min="13" max="13"/>
+    <col width="6" customWidth="1" min="14" max="14"/>
+    <col width="6" customWidth="1" min="15" max="15"/>
+    <col width="6" customWidth="1" min="16" max="16"/>
+    <col width="6" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>2026-10-19 — 8 sectors</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>from \ to</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q3" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL OUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>EBB</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="5" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>BJM</t>
+        </is>
+      </c>
+      <c r="Q5" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>BOM</t>
+        </is>
+      </c>
+      <c r="Q6" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>DAR</t>
+        </is>
+      </c>
+      <c r="Q7" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>HRE</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>JNB</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>JRO</t>
+        </is>
+      </c>
+      <c r="Q10" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>JUB</t>
+        </is>
+      </c>
+      <c r="Q11" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>LGW</t>
+        </is>
+      </c>
+      <c r="Q12" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>LOS</t>
+        </is>
+      </c>
+      <c r="Q13" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>LUN</t>
+        </is>
+      </c>
+      <c r="Q14" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>MBA</t>
+        </is>
+      </c>
+      <c r="Q15" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>MGQ</t>
+        </is>
+      </c>
+      <c r="Q16" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>NBO</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>ZNZ</t>
+        </is>
+      </c>
+      <c r="Q18" s="5" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL IN</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>4</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="L19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O19" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="5" t="n">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -11546,7 +12316,7 @@
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>October 2026 (1-18 Oct) — all sectors</t>
+          <t>October 2026 (1-19 Oct) — all sectors</t>
         </is>
       </c>
     </row>
@@ -11644,7 +12414,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D4" s="4" t="n">
         <v>5</v>
@@ -11656,34 +12426,34 @@
         <v>10</v>
       </c>
       <c r="G4" s="4" t="n">
+        <v>21</v>
+      </c>
+      <c r="I4" s="4" t="n">
         <v>19</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>17</v>
       </c>
       <c r="J4" s="4" t="n">
         <v>8</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>11</v>
       </c>
-      <c r="L4" s="4" t="n">
-        <v>10</v>
-      </c>
       <c r="M4" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N4" s="4" t="n">
         <v>10</v>
       </c>
       <c r="O4" s="4" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="P4" s="4" t="n">
         <v>8</v>
       </c>
       <c r="Q4" s="5" t="n">
-        <v>175</v>
+        <v>186</v>
       </c>
     </row>
     <row r="5">
@@ -11693,10 +12463,10 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="Q5" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="6">
@@ -11719,13 +12489,13 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="O7" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q7" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="8">
@@ -11735,13 +12505,13 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="L8" s="4" t="n">
         <v>6</v>
       </c>
       <c r="Q8" s="5" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -11751,10 +12521,10 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="Q9" s="5" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
@@ -11764,10 +12534,10 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Q10" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
@@ -11777,13 +12547,13 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="O11" s="4" t="n">
         <v>1</v>
       </c>
       <c r="Q11" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="12">
@@ -11793,10 +12563,10 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q12" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13">
@@ -11806,10 +12576,10 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="Q13" s="5" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="14">
@@ -11835,10 +12605,10 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Q15" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">
@@ -11848,10 +12618,10 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="Q16" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="17">
@@ -11861,10 +12631,10 @@
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="Q17" s="5" t="n">
-        <v>39</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18">
@@ -11887,10 +12657,10 @@
         </is>
       </c>
       <c r="B19" s="5" t="n">
-        <v>169</v>
+        <v>183</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D19" s="5" t="n">
         <v>5</v>
@@ -11902,37 +12672,37 @@
         <v>13</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="H19" s="5" t="n">
         <v>5</v>
       </c>
       <c r="I19" s="5" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="J19" s="5" t="n">
         <v>8</v>
       </c>
       <c r="K19" s="5" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="L19" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="M19" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="N19" s="5" t="n">
         <v>10</v>
       </c>
       <c r="O19" s="5" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="P19" s="5" t="n">
         <v>8</v>
       </c>
       <c r="Q19" s="5" t="n">
-        <v>360</v>
+        <v>385</v>
       </c>
     </row>
   </sheetData>

</xml_diff>